<commit_message>
docs: actualizar HU y arquitectura con nombres atomizados, facturas múltiples y devolución de saldo
</commit_message>
<xml_diff>
--- a/docs/EduSaldo - Plantilla Gestión Requerimientos.xlsx
+++ b/docs/EduSaldo - Plantilla Gestión Requerimientos.xlsx
@@ -1398,6 +1398,66 @@
   <si>
     <t>Fusiona ex-HU50 y ex-HU53. Regla: 1 factura por recepción; rechazo puntual de recepción/factura manteniendo la OC vigente; múltiples recepciones/facturas por OC.</t>
   </si>
+  <si>
+    <t>CA1: Dado el formulario, cuando ingresa primer nombre, primer apellido, correo y mensaje válidos (segundo nombre y segundo apellido opcionales), entonces la consulta queda registrada o confirmada para envío. CA2: Dado datos inválidos, cuando intenta enviar, entonces el sistema informa los errores y no procesa la consulta.</t>
+  </si>
+  <si>
+    <t>Nombres atomizados en formulario de consulta.</t>
+  </si>
+  <si>
+    <t>CA1: Dado datos válidos de RUT, primer nombre, segundo nombre (opcional), primer apellido, segundo apellido (opcional), correo y rol, cuando el Administrador confirma, entonces se crea el usuario con contraseña temporal y PRIMER_ACCESO. CA2: Dado el rol seleccionado, cuando el usuario inicia sesión, entonces solo accede a las funciones autorizadas. CA3: Dado la creación, cuando se genera la contraseña temporal, entonces no se almacena ni expone en texto plano.</t>
+  </si>
+  <si>
+    <t>Nombres atomizados para usuarios de staff.</t>
+  </si>
+  <si>
+    <t>CA1: Dado un alumno nuevo con RUT válido y único, primer nombre, segundo nombre (opcional), primer apellido, segundo apellido (opcional), fecha de nacimiento y curso, cuando el Administrador ingresa además los datos de un apoderado y su parentesco y confirma, entonces se crean el alumno en estado ACTIVO y la asociación apoderado-alumno en una sola operación. CA2: Dado un RUT de apoderado que no existe, cuando se confirma el alta, entonces se crea el usuario Apoderado con contraseña temporal y estado PRIMER_ACCESO. CA3: Dado un RUT de apoderado ya registrado, cuando se confirma el alta, entonces se reutiliza ese usuario y solo se crea la nueva asociación. CA4: Dado un RUT de alumno ya registrado o datos de alumno o apoderado inválidos, cuando intenta confirmar, entonces el sistema impide el alta y no crea ningún registro. CA5: Dado un fallo al crear el usuario Apoderado, cuando no puede completarse el alta, entonces no queda un alumno sin apoderado ni un apoderado sin alumno. CA6: Dado los datos del apoderado, cuando se ingresan, entonces se registran por separado primer nombre, segundo nombre (opcional), primer apellido y segundo apellido (opcional).</t>
+  </si>
+  <si>
+    <t>Fusiona ex-HU04 (creación de apoderado). Asociación obligatoria. Nombres atomizados para alumno y apoderado.</t>
+  </si>
+  <si>
+    <t>CA1: Dado un alumno con reservas pendientes o saldo por resolver, cuando se intenta inactivar, entonces el sistema advierte las situaciones pendientes. CA2: Dado un alumno INACTIVO, cuando se consulta desde la cuenta de su apoderado, entonces no permite nuevos abonos, reservas ni compras. CA3: Dada una cuenta de apoderado sin alumnos activos, cuando el Administrador lo decide, entonces puede inactivar también la cuenta. CA4: Dado un alumno inactivado, cuando se consulta su historial, entonces sus asociaciones con apoderados se conservan. CA5: Dado un alumno con saldo disponible y sin reservas pendientes, cuando el Administrador registra la devolución de saldo indicando apoderado receptor, monto, medio (efectivo o transferencia), comprobante y motivo, entonces el saldo del alumno queda en cero con un movimiento DEVOLUCION_SALDO y se genera un único egreso en la Cuenta Librería. CA6: Dado un alumno con reservas pendientes, cuando se intenta registrar la devolución de saldo, entonces el sistema lo impide hasta cancelar o entregar esas reservas. CA7: Dado la devolución, cuando se registra, entonces la entrega física del dinero se realiza fuera del sistema y la operación queda auditada.</t>
+  </si>
+  <si>
+    <t>Agrega CA4: se conservan las asociaciones con apoderados. Agrega devolución de saldo (retiro o cambio de colegio): entrega manual, registro obligatorio.</t>
+  </si>
+  <si>
+    <t>CA1: Dado un Apoderado autenticado, cuando ingresa a Mis alumnos, entonces solo visualiza los alumnos asociados a su cuenta. CA2: Dado cada alumno, cuando se muestra, entonces visualiza su nombre completo (compuesto desde primer nombre, segundo nombre, primer apellido y segundo apellido), curso y RUT enmascarado. CA3: Dado alumnos inactivos con historial, cuando corresponda, entonces se muestran solo para consulta histórica y sin acciones nuevas.</t>
+  </si>
+  <si>
+    <t>Nombre completo compuesto desde campos atomizados.</t>
+  </si>
+  <si>
+    <t>CA1: Dado un proveedor válido, cuando se registra, entonces queda disponible para nuevas órdenes de compra. CA2: Dado un proveedor con historial, cuando deja de utilizarse, entonces se inactiva sin eliminar sus compras anteriores. CA3: Dado el contacto del proveedor, cuando se registra, entonces se guardan por separado primer nombre, segundo nombre (opcional), primer apellido, segundo apellido (opcional), correo y teléfono.</t>
+  </si>
+  <si>
+    <t>Contacto del proveedor con nombre atomizado.</t>
+  </si>
+  <si>
+    <t>Registrar la recepción de mercadería con sus facturas</t>
+  </si>
+  <si>
+    <t>ingresar al stock solo mercadería respaldada por facturas que coinciden</t>
+  </si>
+  <si>
+    <t>CA1: Dado una OC vigente, cuando llega mercadería con una o más facturas, entonces el Encargado registra cada factura (número, fecha, neto, IVA, total y sus líneas de producto, entre 1 y 60) y compara producto y cantidad contra la OC y las facturas. CA2: Dado que la suma de las cantidades facturadas por producto coincide exactamente con lo recibido, cuando confirma, entonces la recepción queda ACEPTADA como COMPLETA o INCOMPLETA, aumenta el stock físico por las unidades recibidas y se recalcula el CPP. CA3: Dado que las facturas no coinciden con la mercadería recibida o contienen artículos no ordenados, cuando se revisa, entonces la recepción puntual queda RECHAZADA con motivo obligatorio (junto con todas sus facturas), no modifica stock ni CPP, y la OC permanece vigente para un nuevo despacho. CA4: Dado una recepción INCOMPLETA aceptada, cuando quedan unidades pendientes, entonces la OC queda en RECEPCIÓN_PARCIAL y abierta para nuevas recepciones. CA5: Dado una OC con varias recepciones, cuando se consulta, entonces cada recepción muestra sus facturas, y cada factura aceptada queda pendiente de pago en Finanzas (se paga completa, sin pagos parciales).</t>
+  </si>
+  <si>
+    <t>Fusiona ex-HU50 y ex-HU53. Regla: 1 factura por recepción; rechazo puntual de recepción/factura manteniendo la OC vigente; múltiples recepciones/facturas por OC. Una recepción puede traer 1..* facturas (p. ej. límite de 60 ítems por factura del SII).</t>
+  </si>
+  <si>
+    <t>CA1: Dado movimientos financieros, cuando se consulta la cartola, entonces muestra fecha, tipo, referencia, monto y saldo. CA2: Dado el rol Autorizador, cuando consulta, entonces el acceso es de solo lectura salvo sus acciones de autorización. CA3: Dado abonos, pagos de facturas y devoluciones de saldo, cuando se registran, entonces aparecen una sola vez en la cartola y no se duplican por la venta/consumo del saldo.</t>
+  </si>
+  <si>
+    <t>Registra devoluciones de saldo en cartola de caja.</t>
+  </si>
+  <si>
+    <t>CA1: Dado un rango de fechas, cuando consulta reportes, entonces puede visualizar abonos, consumos/ventas, devoluciones de venta, devoluciones de saldo, pagos y otros indicadores definidos. CA2: Dado reportes, cuando se muestran, entonces distinguen movimientos de saldo de movimientos de caja para evitar doble contabilización. CA3: Dado información disponible, cuando se solicita, entonces se presentan gráficos/resúmenes sin alterar los datos fuente.</t>
+  </si>
+  <si>
+    <t>Distingue devoluciones de venta y de saldo en reportes.</t>
+  </si>
 </sst>
 </file>
 
@@ -29260,13 +29320,15 @@
         <v>42</v>
       </c>
       <c r="I4" s="4" t="s">
-        <v>67</v>
+        <v>456</v>
       </c>
       <c r="J4" s="4" t="s">
         <v>17</v>
       </c>
       <c r="K4" s="4"/>
-      <c r="L4" s="4"/>
+      <c r="L4" s="4" t="s">
+        <v>457</v>
+      </c>
       <c r="M4" s="6"/>
       <c r="N4" s="6"/>
       <c r="O4" s="6"/>
@@ -29303,13 +29365,15 @@
         <v>42</v>
       </c>
       <c r="I5" s="4" t="s">
-        <v>74</v>
+        <v>458</v>
       </c>
       <c r="J5" s="4" t="s">
         <v>17</v>
       </c>
       <c r="K5" s="4"/>
-      <c r="L5" s="4"/>
+      <c r="L5" s="4" t="s">
+        <v>459</v>
+      </c>
       <c r="M5" s="6"/>
       <c r="N5" s="6"/>
       <c r="O5" s="6"/>
@@ -29737,14 +29801,14 @@
         <v>42</v>
       </c>
       <c r="I15" s="4" t="s">
-        <v>417</v>
+        <v>460</v>
       </c>
       <c r="J15" s="4" t="s">
         <v>17</v>
       </c>
       <c r="K15" s="4"/>
       <c r="L15" s="4" t="s">
-        <v>418</v>
+        <v>461</v>
       </c>
       <c r="M15" s="6"/>
       <c r="N15" s="6"/>
@@ -29870,14 +29934,14 @@
         <v>42</v>
       </c>
       <c r="I18" s="4" t="s">
-        <v>425</v>
+        <v>462</v>
       </c>
       <c r="J18" s="4" t="s">
         <v>17</v>
       </c>
       <c r="K18" s="4"/>
       <c r="L18" s="4" t="s">
-        <v>426</v>
+        <v>463</v>
       </c>
       <c r="M18" s="6"/>
       <c r="N18" s="6"/>
@@ -29915,13 +29979,15 @@
         <v>42</v>
       </c>
       <c r="I19" s="4" t="s">
-        <v>138</v>
+        <v>464</v>
       </c>
       <c r="J19" s="4" t="s">
         <v>17</v>
       </c>
       <c r="K19" s="4"/>
-      <c r="L19" s="4"/>
+      <c r="L19" s="4" t="s">
+        <v>465</v>
+      </c>
       <c r="M19" s="6"/>
       <c r="N19" s="6"/>
       <c r="O19" s="6"/>
@@ -31090,13 +31156,15 @@
         <v>42</v>
       </c>
       <c r="I46" s="4" t="s">
-        <v>278</v>
+        <v>466</v>
       </c>
       <c r="J46" s="4" t="s">
         <v>17</v>
       </c>
       <c r="K46" s="4"/>
-      <c r="L46" s="4"/>
+      <c r="L46" s="4" t="s">
+        <v>467</v>
+      </c>
       <c r="M46" s="6"/>
       <c r="N46" s="6"/>
       <c r="O46" s="6"/>
@@ -31203,7 +31271,7 @@
         <v>46</v>
       </c>
       <c r="C49" s="4" t="s">
-        <v>444</v>
+        <v>468</v>
       </c>
       <c r="D49" s="4" t="s">
         <v>192</v>
@@ -31212,7 +31280,7 @@
         <v>445</v>
       </c>
       <c r="F49" s="4" t="s">
-        <v>446</v>
+        <v>469</v>
       </c>
       <c r="G49" s="4" t="s">
         <v>23</v>
@@ -31221,14 +31289,14 @@
         <v>42</v>
       </c>
       <c r="I49" s="4" t="s">
-        <v>454</v>
+        <v>470</v>
       </c>
       <c r="J49" s="4" t="s">
         <v>17</v>
       </c>
       <c r="K49" s="4"/>
       <c r="L49" s="4" t="s">
-        <v>455</v>
+        <v>471</v>
       </c>
       <c r="M49" s="6"/>
       <c r="N49" s="6"/>
@@ -31352,13 +31420,15 @@
         <v>42</v>
       </c>
       <c r="I52" s="4" t="s">
-        <v>319</v>
+        <v>472</v>
       </c>
       <c r="J52" s="4" t="s">
         <v>17</v>
       </c>
       <c r="K52" s="4"/>
-      <c r="L52" s="4"/>
+      <c r="L52" s="4" t="s">
+        <v>473</v>
+      </c>
       <c r="M52" s="6"/>
       <c r="N52" s="6"/>
       <c r="O52" s="6"/>
@@ -31524,13 +31594,15 @@
         <v>42</v>
       </c>
       <c r="I56" s="4" t="s">
-        <v>340</v>
+        <v>474</v>
       </c>
       <c r="J56" s="4" t="s">
         <v>17</v>
       </c>
       <c r="K56" s="4"/>
-      <c r="L56" s="4"/>
+      <c r="L56" s="4" t="s">
+        <v>475</v>
+      </c>
       <c r="M56" s="6"/>
       <c r="N56" s="6"/>
       <c r="O56" s="6"/>

</xml_diff>